<commit_message>
blockwall UI: DEX, Aktien, Einzahlung modal, balance hide, refresh, loader, currency profile
</commit_message>
<xml_diff>
--- a/data/wallets.xlsx
+++ b/data/wallets.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,6 +476,314 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>demo@blockchain-demo.com</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>demo@blockchain-demo.com</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>demo@blockchain-demo.com</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Tether</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>demo@blockchain-demo.com</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>BNB</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>BNB</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>BNB</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>demo@blockchain-demo.com</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>demo@blockchain-demo.com</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>USDC</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>USD Coin</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>USDC</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>demo@blockchain-demo.com</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>demo@blockchain-demo.com</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ADA</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Cardano</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>ADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>demo@blockchain-demo.com</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>DOGE</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Dogecoin</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>DOGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>demo@blockchain-demo.com</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>MATIC</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Polygon</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>MATIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>demo@blockchain-demo.com</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>DOT</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Polkadot</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>DOT</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix migration: swap seed_qty and seed_eur dict sources (was writing qty to eur column)
</commit_message>
<xml_diff>
--- a/data/wallets.xlsx
+++ b/data/wallets.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="wallets" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="wallets" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,6 +447,11 @@
           <t>qty_unit</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>address</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -475,6 +480,11 @@
           <t>TRX</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>TQrZ7d8xNhP9xK2yR5hLkQ3jF8m6bC4wYvE</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -493,14 +503,19 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>2180.8625</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>0.025</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>BTC</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>bc1qxy2kgdygjrsqtzq2n0yrf2493p83kkfjhx0wlh</t>
         </is>
       </c>
     </row>
@@ -531,6 +546,11 @@
           <t>ETH</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0x71C7656EC7ab88b098defB751B7401B5f6d8976F</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -559,6 +579,11 @@
           <t>USDT</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>TR7NHqjeKQxGTCi8q8ZY4pL8otSzgjD6Sz</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -587,6 +612,11 @@
           <t>BNB</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>bnb1grpf0955t0tlt8eaw9g0w78v5q8v3f5d3wqczp</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -615,6 +645,11 @@
           <t>SOL</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>7EYnhQoAGqH7ZbRq8HQq8j4xQ4v5v9NQ7vC2vN3o8X7XJ</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -643,6 +678,11 @@
           <t>USDC</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0xA0b86991c6218b36c1d19D4a2e9Eb0cE3606eB48</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -671,6 +711,11 @@
           <t>XRP</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>rDsbeomae4FXwgQTJp9Rs64Qg9vDiTCdBv</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -699,6 +744,11 @@
           <t>ADA</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>addr1q9zy2kgdygjrsqtzq2n0yrf2493p83kkfjhx0wlh</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -727,6 +777,11 @@
           <t>DOGE</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>DH5yaieqoZN36pDV3xcpbwAY7Sa1YQsv7p</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -755,6 +810,11 @@
           <t>MATIC</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>0x742d35Cc6634C0532925a3b844Bc9e7595f0bEb0</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -781,6 +841,11 @@
       <c r="F13" t="inlineStr">
         <is>
           <t>DOT</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>1FRMM8d8HdJzk6FpZ7j5vW2pGcZ7Y2qJxC8Rf5oKjHn8U</t>
         </is>
       </c>
     </row>

</xml_diff>